<commit_message>
Refactor dashboard flow and add enrolment view
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://depedph-my.sharepoint.com/personal/eloisa_baylon_deped_gov_ph/Documents/Desktop/JASON_FILE/web/ALS_PROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{CDD84AC6-4E25-4955-92B4-7194A5FDD9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7145760B-CEB7-4D3C-8B26-DFB6E1A9C246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{22E19479-EE82-45A3-9220-E5159A49DAD2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{22E19479-EE82-45A3-9220-E5159A49DAD2}"/>
   </bookViews>
   <sheets>
     <sheet name="divisions" sheetId="1" r:id="rId1"/>
     <sheet name="teachers" sheetId="2" r:id="rId2"/>
     <sheet name="schools" sheetId="3" r:id="rId3"/>
+    <sheet name="enrolment" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="463">
   <si>
     <t>id</t>
   </si>
@@ -1349,13 +1350,91 @@
   </si>
   <si>
     <t>OCAMPO, ROME NIKEY, PARAGAS</t>
+  </si>
+  <si>
+    <t>Division</t>
+  </si>
+  <si>
+    <t>Basic Literacy Program</t>
+  </si>
+  <si>
+    <t>A&amp;E Elementary</t>
+  </si>
+  <si>
+    <t>A&amp;E Junior High School</t>
+  </si>
+  <si>
+    <t>BP-OSA - Mandaluyong only</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Caloocan</t>
+  </si>
+  <si>
+    <t>Las Piñas</t>
+  </si>
+  <si>
+    <t>Makati</t>
+  </si>
+  <si>
+    <t>Malabon</t>
+  </si>
+  <si>
+    <t>Mandaluyong</t>
+  </si>
+  <si>
+    <t>Manila</t>
+  </si>
+  <si>
+    <t>Marikina</t>
+  </si>
+  <si>
+    <t>Muntinlupa</t>
+  </si>
+  <si>
+    <t>Navotas</t>
+  </si>
+  <si>
+    <t>Parañaque</t>
+  </si>
+  <si>
+    <t>Pasay</t>
+  </si>
+  <si>
+    <t>Pasig</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Quezon City</t>
+  </si>
+  <si>
+    <t>San Juan</t>
+  </si>
+  <si>
+    <t>TaPat</t>
+  </si>
+  <si>
+    <t>Valenzuela</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1417,6 +1496,29 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1432,7 +1534,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1468,11 +1570,104 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1519,6 +1714,36 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7669,4 +7894,940 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90C2FF11-C04B-4FC3-A426-A14BD7863204}">
+  <dimension ref="A1:P19"/>
+  <sheetFormatPr defaultColWidth="15.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="C1" s="22"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="21" t="s">
+        <v>439</v>
+      </c>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="I1" s="22"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="L1" s="22"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="O1" s="22"/>
+      <c r="P1" s="23"/>
+    </row>
+    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="24"/>
+      <c r="B2" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>444</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>445</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>444</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>445</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>444</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>445</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="L2" s="25" t="s">
+        <v>444</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>445</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="O2" s="25" t="s">
+        <v>444</v>
+      </c>
+      <c r="P2" s="25" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="26" t="s">
+        <v>446</v>
+      </c>
+      <c r="B3" s="25">
+        <v>43</v>
+      </c>
+      <c r="C3" s="25">
+        <v>15</v>
+      </c>
+      <c r="D3" s="25">
+        <v>58</v>
+      </c>
+      <c r="E3" s="25">
+        <v>496</v>
+      </c>
+      <c r="F3" s="25">
+        <v>288</v>
+      </c>
+      <c r="G3" s="25">
+        <v>784</v>
+      </c>
+      <c r="H3" s="25">
+        <v>1399</v>
+      </c>
+      <c r="I3" s="25">
+        <v>1207</v>
+      </c>
+      <c r="J3" s="25">
+        <v>2606</v>
+      </c>
+      <c r="K3" s="25">
+        <v>0</v>
+      </c>
+      <c r="L3" s="25">
+        <v>0</v>
+      </c>
+      <c r="M3" s="25">
+        <v>0</v>
+      </c>
+      <c r="N3" s="25">
+        <v>1938</v>
+      </c>
+      <c r="O3" s="25">
+        <v>1510</v>
+      </c>
+      <c r="P3" s="25">
+        <v>3448</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="26" t="s">
+        <v>447</v>
+      </c>
+      <c r="B4" s="25">
+        <v>22</v>
+      </c>
+      <c r="C4" s="25">
+        <v>13</v>
+      </c>
+      <c r="D4" s="25">
+        <v>35</v>
+      </c>
+      <c r="E4" s="25">
+        <v>252</v>
+      </c>
+      <c r="F4" s="25">
+        <v>110</v>
+      </c>
+      <c r="G4" s="25">
+        <v>362</v>
+      </c>
+      <c r="H4" s="25">
+        <v>706</v>
+      </c>
+      <c r="I4" s="25">
+        <v>390</v>
+      </c>
+      <c r="J4" s="25">
+        <v>1096</v>
+      </c>
+      <c r="K4" s="25">
+        <v>0</v>
+      </c>
+      <c r="L4" s="25">
+        <v>0</v>
+      </c>
+      <c r="M4" s="25">
+        <v>0</v>
+      </c>
+      <c r="N4" s="25">
+        <v>980</v>
+      </c>
+      <c r="O4" s="25">
+        <v>513</v>
+      </c>
+      <c r="P4" s="25">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="26" t="s">
+        <v>448</v>
+      </c>
+      <c r="B5" s="25">
+        <v>27</v>
+      </c>
+      <c r="C5" s="25">
+        <v>9</v>
+      </c>
+      <c r="D5" s="25">
+        <v>36</v>
+      </c>
+      <c r="E5" s="25">
+        <v>116</v>
+      </c>
+      <c r="F5" s="25">
+        <v>182</v>
+      </c>
+      <c r="G5" s="25">
+        <v>298</v>
+      </c>
+      <c r="H5" s="25">
+        <v>249</v>
+      </c>
+      <c r="I5" s="25">
+        <v>175</v>
+      </c>
+      <c r="J5" s="25">
+        <v>424</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="25">
+        <v>392</v>
+      </c>
+      <c r="O5" s="25">
+        <v>366</v>
+      </c>
+      <c r="P5" s="25">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="B6" s="25">
+        <v>20</v>
+      </c>
+      <c r="C6" s="25">
+        <v>9</v>
+      </c>
+      <c r="D6" s="25">
+        <v>29</v>
+      </c>
+      <c r="E6" s="25">
+        <v>97</v>
+      </c>
+      <c r="F6" s="25">
+        <v>62</v>
+      </c>
+      <c r="G6" s="25">
+        <v>159</v>
+      </c>
+      <c r="H6" s="25">
+        <v>185</v>
+      </c>
+      <c r="I6" s="25">
+        <v>168</v>
+      </c>
+      <c r="J6" s="25">
+        <v>353</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="25">
+        <v>302</v>
+      </c>
+      <c r="O6" s="25">
+        <v>239</v>
+      </c>
+      <c r="P6" s="25">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="26" t="s">
+        <v>450</v>
+      </c>
+      <c r="B7" s="25">
+        <v>20</v>
+      </c>
+      <c r="C7" s="25">
+        <v>45</v>
+      </c>
+      <c r="D7" s="25">
+        <v>65</v>
+      </c>
+      <c r="E7" s="25">
+        <v>139</v>
+      </c>
+      <c r="F7" s="25">
+        <v>83</v>
+      </c>
+      <c r="G7" s="25">
+        <v>222</v>
+      </c>
+      <c r="H7" s="25">
+        <v>525</v>
+      </c>
+      <c r="I7" s="25">
+        <v>384</v>
+      </c>
+      <c r="J7" s="25">
+        <v>909</v>
+      </c>
+      <c r="K7" s="25">
+        <v>143</v>
+      </c>
+      <c r="L7" s="25">
+        <v>91</v>
+      </c>
+      <c r="M7" s="25">
+        <v>234</v>
+      </c>
+      <c r="N7" s="25">
+        <v>827</v>
+      </c>
+      <c r="O7" s="25">
+        <v>603</v>
+      </c>
+      <c r="P7" s="25">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="26" t="s">
+        <v>451</v>
+      </c>
+      <c r="B8" s="25">
+        <v>71</v>
+      </c>
+      <c r="C8" s="25">
+        <v>63</v>
+      </c>
+      <c r="D8" s="25">
+        <v>134</v>
+      </c>
+      <c r="E8" s="25">
+        <v>1358</v>
+      </c>
+      <c r="F8" s="25">
+        <v>872</v>
+      </c>
+      <c r="G8" s="25">
+        <v>2230</v>
+      </c>
+      <c r="H8" s="25">
+        <v>2470</v>
+      </c>
+      <c r="I8" s="25">
+        <v>1862</v>
+      </c>
+      <c r="J8" s="25">
+        <v>4332</v>
+      </c>
+      <c r="K8" s="25">
+        <v>0</v>
+      </c>
+      <c r="L8" s="25">
+        <v>0</v>
+      </c>
+      <c r="M8" s="25">
+        <v>0</v>
+      </c>
+      <c r="N8" s="25">
+        <v>3899</v>
+      </c>
+      <c r="O8" s="25">
+        <v>2797</v>
+      </c>
+      <c r="P8" s="25">
+        <v>6696</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="26" t="s">
+        <v>452</v>
+      </c>
+      <c r="B9" s="25">
+        <v>2</v>
+      </c>
+      <c r="C9" s="25">
+        <v>2</v>
+      </c>
+      <c r="D9" s="25">
+        <v>4</v>
+      </c>
+      <c r="E9" s="25">
+        <v>99</v>
+      </c>
+      <c r="F9" s="25">
+        <v>63</v>
+      </c>
+      <c r="G9" s="25">
+        <v>162</v>
+      </c>
+      <c r="H9" s="25">
+        <v>330</v>
+      </c>
+      <c r="I9" s="25">
+        <v>232</v>
+      </c>
+      <c r="J9" s="25">
+        <v>562</v>
+      </c>
+      <c r="K9" s="25">
+        <v>0</v>
+      </c>
+      <c r="L9" s="25">
+        <v>0</v>
+      </c>
+      <c r="M9" s="25">
+        <v>0</v>
+      </c>
+      <c r="N9" s="25">
+        <v>431</v>
+      </c>
+      <c r="O9" s="25">
+        <v>297</v>
+      </c>
+      <c r="P9" s="25">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="26" t="s">
+        <v>453</v>
+      </c>
+      <c r="B10" s="25">
+        <v>282</v>
+      </c>
+      <c r="C10" s="25">
+        <v>10</v>
+      </c>
+      <c r="D10" s="25">
+        <v>292</v>
+      </c>
+      <c r="E10" s="25">
+        <v>793</v>
+      </c>
+      <c r="F10" s="25">
+        <v>90</v>
+      </c>
+      <c r="G10" s="25">
+        <v>883</v>
+      </c>
+      <c r="H10" s="25">
+        <v>1331</v>
+      </c>
+      <c r="I10" s="25">
+        <v>384</v>
+      </c>
+      <c r="J10" s="25">
+        <v>1715</v>
+      </c>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="25">
+        <v>0</v>
+      </c>
+      <c r="N10" s="25">
+        <v>2406</v>
+      </c>
+      <c r="O10" s="25">
+        <v>484</v>
+      </c>
+      <c r="P10" s="25">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="26" t="s">
+        <v>454</v>
+      </c>
+      <c r="B11" s="25">
+        <v>37</v>
+      </c>
+      <c r="C11" s="25">
+        <v>12</v>
+      </c>
+      <c r="D11" s="25">
+        <v>49</v>
+      </c>
+      <c r="E11" s="25">
+        <v>134</v>
+      </c>
+      <c r="F11" s="25">
+        <v>79</v>
+      </c>
+      <c r="G11" s="25">
+        <v>213</v>
+      </c>
+      <c r="H11" s="25">
+        <v>249</v>
+      </c>
+      <c r="I11" s="25">
+        <v>214</v>
+      </c>
+      <c r="J11" s="25">
+        <v>463</v>
+      </c>
+      <c r="K11" s="25">
+        <v>0</v>
+      </c>
+      <c r="L11" s="25">
+        <v>0</v>
+      </c>
+      <c r="M11" s="25">
+        <v>0</v>
+      </c>
+      <c r="N11" s="25">
+        <v>420</v>
+      </c>
+      <c r="O11" s="25">
+        <v>305</v>
+      </c>
+      <c r="P11" s="25">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="26" t="s">
+        <v>455</v>
+      </c>
+      <c r="B12" s="25">
+        <v>14</v>
+      </c>
+      <c r="C12" s="25">
+        <v>11</v>
+      </c>
+      <c r="D12" s="25">
+        <v>25</v>
+      </c>
+      <c r="E12" s="25">
+        <v>163</v>
+      </c>
+      <c r="F12" s="25">
+        <v>130</v>
+      </c>
+      <c r="G12" s="25">
+        <v>293</v>
+      </c>
+      <c r="H12" s="25">
+        <v>463</v>
+      </c>
+      <c r="I12" s="25">
+        <v>493</v>
+      </c>
+      <c r="J12" s="25">
+        <v>956</v>
+      </c>
+      <c r="K12" s="25">
+        <v>0</v>
+      </c>
+      <c r="L12" s="25">
+        <v>0</v>
+      </c>
+      <c r="M12" s="25">
+        <v>0</v>
+      </c>
+      <c r="N12" s="25">
+        <v>640</v>
+      </c>
+      <c r="O12" s="25">
+        <v>634</v>
+      </c>
+      <c r="P12" s="25">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="26" t="s">
+        <v>456</v>
+      </c>
+      <c r="B13" s="25">
+        <v>85</v>
+      </c>
+      <c r="C13" s="25">
+        <v>24</v>
+      </c>
+      <c r="D13" s="25">
+        <v>109</v>
+      </c>
+      <c r="E13" s="25">
+        <v>185</v>
+      </c>
+      <c r="F13" s="25">
+        <v>130</v>
+      </c>
+      <c r="G13" s="25">
+        <v>315</v>
+      </c>
+      <c r="H13" s="25">
+        <v>528</v>
+      </c>
+      <c r="I13" s="25">
+        <v>629</v>
+      </c>
+      <c r="J13" s="25">
+        <v>1157</v>
+      </c>
+      <c r="K13" s="25">
+        <v>0</v>
+      </c>
+      <c r="L13" s="25">
+        <v>0</v>
+      </c>
+      <c r="M13" s="25">
+        <v>0</v>
+      </c>
+      <c r="N13" s="25">
+        <v>798</v>
+      </c>
+      <c r="O13" s="25">
+        <v>783</v>
+      </c>
+      <c r="P13" s="25">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="26" t="s">
+        <v>457</v>
+      </c>
+      <c r="B14" s="25">
+        <v>15</v>
+      </c>
+      <c r="C14" s="25">
+        <v>11</v>
+      </c>
+      <c r="D14" s="25">
+        <v>26</v>
+      </c>
+      <c r="E14" s="25">
+        <v>146</v>
+      </c>
+      <c r="F14" s="25">
+        <v>64</v>
+      </c>
+      <c r="G14" s="25">
+        <v>210</v>
+      </c>
+      <c r="H14" s="25">
+        <v>687</v>
+      </c>
+      <c r="I14" s="25">
+        <v>436</v>
+      </c>
+      <c r="J14" s="25">
+        <v>1123</v>
+      </c>
+      <c r="K14" s="25" t="s">
+        <v>458</v>
+      </c>
+      <c r="L14" s="25" t="s">
+        <v>458</v>
+      </c>
+      <c r="M14" s="25">
+        <v>0</v>
+      </c>
+      <c r="N14" s="25">
+        <v>848</v>
+      </c>
+      <c r="O14" s="25">
+        <v>511</v>
+      </c>
+      <c r="P14" s="25">
+        <v>1359</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="26" t="s">
+        <v>459</v>
+      </c>
+      <c r="B15" s="25">
+        <v>74</v>
+      </c>
+      <c r="C15" s="25">
+        <v>36</v>
+      </c>
+      <c r="D15" s="25">
+        <v>110</v>
+      </c>
+      <c r="E15" s="25">
+        <v>527</v>
+      </c>
+      <c r="F15" s="25">
+        <v>260</v>
+      </c>
+      <c r="G15" s="25">
+        <v>787</v>
+      </c>
+      <c r="H15" s="25">
+        <v>1782</v>
+      </c>
+      <c r="I15" s="25">
+        <v>1240</v>
+      </c>
+      <c r="J15" s="25">
+        <v>3022</v>
+      </c>
+      <c r="K15" s="25">
+        <v>0</v>
+      </c>
+      <c r="L15" s="25">
+        <v>0</v>
+      </c>
+      <c r="M15" s="25">
+        <v>0</v>
+      </c>
+      <c r="N15" s="25">
+        <v>2383</v>
+      </c>
+      <c r="O15" s="25">
+        <v>1536</v>
+      </c>
+      <c r="P15" s="25">
+        <v>3919</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="26" t="s">
+        <v>460</v>
+      </c>
+      <c r="B16" s="25">
+        <v>4</v>
+      </c>
+      <c r="C16" s="25">
+        <v>6</v>
+      </c>
+      <c r="D16" s="25">
+        <v>10</v>
+      </c>
+      <c r="E16" s="25">
+        <v>28</v>
+      </c>
+      <c r="F16" s="25">
+        <v>19</v>
+      </c>
+      <c r="G16" s="25">
+        <v>47</v>
+      </c>
+      <c r="H16" s="25">
+        <v>100</v>
+      </c>
+      <c r="I16" s="25">
+        <v>69</v>
+      </c>
+      <c r="J16" s="25">
+        <v>169</v>
+      </c>
+      <c r="K16" s="25">
+        <v>0</v>
+      </c>
+      <c r="L16" s="25">
+        <v>0</v>
+      </c>
+      <c r="M16" s="25">
+        <v>0</v>
+      </c>
+      <c r="N16" s="25">
+        <v>132</v>
+      </c>
+      <c r="O16" s="25">
+        <v>94</v>
+      </c>
+      <c r="P16" s="25">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="26" t="s">
+        <v>461</v>
+      </c>
+      <c r="B17" s="25">
+        <v>30</v>
+      </c>
+      <c r="C17" s="25">
+        <v>22</v>
+      </c>
+      <c r="D17" s="25">
+        <v>52</v>
+      </c>
+      <c r="E17" s="25">
+        <v>393</v>
+      </c>
+      <c r="F17" s="25">
+        <v>209</v>
+      </c>
+      <c r="G17" s="25">
+        <v>602</v>
+      </c>
+      <c r="H17" s="25">
+        <v>1269</v>
+      </c>
+      <c r="I17" s="25">
+        <v>898</v>
+      </c>
+      <c r="J17" s="25">
+        <v>2167</v>
+      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="25">
+        <v>0</v>
+      </c>
+      <c r="N17" s="25">
+        <v>1692</v>
+      </c>
+      <c r="O17" s="25">
+        <v>1129</v>
+      </c>
+      <c r="P17" s="25">
+        <v>2821</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="26" t="s">
+        <v>462</v>
+      </c>
+      <c r="B18" s="25">
+        <v>20</v>
+      </c>
+      <c r="C18" s="25">
+        <v>15</v>
+      </c>
+      <c r="D18" s="25">
+        <v>35</v>
+      </c>
+      <c r="E18" s="25">
+        <v>110</v>
+      </c>
+      <c r="F18" s="25">
+        <v>65</v>
+      </c>
+      <c r="G18" s="25">
+        <v>175</v>
+      </c>
+      <c r="H18" s="25">
+        <v>466</v>
+      </c>
+      <c r="I18" s="25">
+        <v>284</v>
+      </c>
+      <c r="J18" s="25">
+        <v>750</v>
+      </c>
+      <c r="K18" s="25">
+        <v>0</v>
+      </c>
+      <c r="L18" s="25">
+        <v>0</v>
+      </c>
+      <c r="M18" s="25">
+        <v>0</v>
+      </c>
+      <c r="N18" s="25">
+        <v>596</v>
+      </c>
+      <c r="O18" s="25">
+        <v>364</v>
+      </c>
+      <c r="P18" s="25">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="28"/>
+      <c r="B19" s="29">
+        <v>766</v>
+      </c>
+      <c r="C19" s="29">
+        <v>303</v>
+      </c>
+      <c r="D19" s="29">
+        <v>1069</v>
+      </c>
+      <c r="E19" s="29">
+        <v>5036</v>
+      </c>
+      <c r="F19" s="29">
+        <v>2706</v>
+      </c>
+      <c r="G19" s="29">
+        <v>7742</v>
+      </c>
+      <c r="H19" s="29">
+        <v>12739</v>
+      </c>
+      <c r="I19" s="29">
+        <v>9065</v>
+      </c>
+      <c r="J19" s="29">
+        <v>21804</v>
+      </c>
+      <c r="K19" s="29">
+        <v>143</v>
+      </c>
+      <c r="L19" s="29">
+        <v>91</v>
+      </c>
+      <c r="M19" s="29">
+        <v>234</v>
+      </c>
+      <c r="N19" s="29">
+        <v>18684</v>
+      </c>
+      <c r="O19" s="29">
+        <v>12165</v>
+      </c>
+      <c r="P19" s="29">
+        <v>30849</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>